<commit_message>
Fix #44 - restored dropdowns and VLOOKUPs after real data import, updated import script to preserve them
- Supply col B: VLOOKUP(A,'Employee Master'!A:B,2,FALSE) on every data row
- Supply col C: Skill Set dropdown from Skills Master
- Supply col D: Project Assigned dropdown from Project Master
- Demand col A: Project dropdown from Project Master
- Demand col B: Resource Level dropdown from Resource Levels
- Demand col C: Skill Set dropdown from Skills Master

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/resourcing.xlsx
+++ b/data/resourcing.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="356" uniqueCount="133">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="312" uniqueCount="133">
   <si>
     <t>Employee Name</t>
   </si>
@@ -72,262 +72,262 @@
     <t>Abdesattar Karim</t>
   </si>
   <si>
+    <t>NetSuite - Record to Report</t>
+  </si>
+  <si>
+    <t>Bank Integration</t>
+  </si>
+  <si>
+    <t>P2P</t>
+  </si>
+  <si>
+    <t>Benjamin Liu</t>
+  </si>
+  <si>
+    <t>NetSuite - Procure to Pay</t>
+  </si>
+  <si>
+    <t>Accounting</t>
+  </si>
+  <si>
+    <t>R2R</t>
+  </si>
+  <si>
+    <t>Christine Chen</t>
+  </si>
+  <si>
+    <t>NetSuite - Order to Cash</t>
+  </si>
+  <si>
+    <t>NetSuite Implementation</t>
+  </si>
+  <si>
+    <t>Crystal Brent</t>
+  </si>
+  <si>
+    <t>NetSuite - Supply Chain</t>
+  </si>
+  <si>
+    <t>Delaney O'Neil</t>
+  </si>
+  <si>
+    <t>Pigment</t>
+  </si>
+  <si>
+    <t>Unassigned</t>
+  </si>
+  <si>
+    <t>Ethan Osborne</t>
+  </si>
+  <si>
+    <t>Phase 0</t>
+  </si>
+  <si>
+    <t>Grace Schwieters</t>
+  </si>
+  <si>
+    <t>Phase 1</t>
+  </si>
+  <si>
+    <t>Phase 0 Design</t>
+  </si>
+  <si>
+    <t>Hannah Imhoff</t>
+  </si>
+  <si>
+    <t>NS Implementation</t>
+  </si>
+  <si>
+    <t>O2C Analyst</t>
+  </si>
+  <si>
+    <t>Jake Johnsen</t>
+  </si>
+  <si>
+    <t>Julie Loiben</t>
+  </si>
+  <si>
+    <t>Flare</t>
+  </si>
+  <si>
+    <t>Katharine Yu</t>
+  </si>
+  <si>
+    <t>Lance Falk</t>
+  </si>
+  <si>
+    <t>Grub WBS</t>
+  </si>
+  <si>
+    <t>Lexie Dutch</t>
+  </si>
+  <si>
+    <t>Marcy Minnerly</t>
+  </si>
+  <si>
+    <t>Secondment</t>
+  </si>
+  <si>
+    <t>Mario DeFelice</t>
+  </si>
+  <si>
+    <t>Evaluation</t>
+  </si>
+  <si>
+    <t>ERP Evaluation</t>
+  </si>
+  <si>
+    <t>Melissa Cross</t>
+  </si>
+  <si>
+    <t>L2C Assessment</t>
+  </si>
+  <si>
+    <t>Assessment</t>
+  </si>
+  <si>
+    <t>Melissa Leighton</t>
+  </si>
+  <si>
+    <t>Neeraj Rajendran</t>
+  </si>
+  <si>
+    <t>Sui Foundation</t>
+  </si>
+  <si>
+    <t>Nick Hernandez</t>
+  </si>
+  <si>
+    <t>Nick Kolbow</t>
+  </si>
+  <si>
+    <t>Ryan Artz</t>
+  </si>
+  <si>
+    <t>Arevon</t>
+  </si>
+  <si>
+    <t>BlankStreet Advisory</t>
+  </si>
+  <si>
+    <t>Procore Advisory</t>
+  </si>
+  <si>
+    <t>Operate</t>
+  </si>
+  <si>
+    <t>Sammy Latif</t>
+  </si>
+  <si>
+    <t>Shreyas Sampath</t>
+  </si>
+  <si>
+    <t>SuiteBilling Implementation</t>
+  </si>
+  <si>
+    <t>SuiteProjects Advisory</t>
+  </si>
+  <si>
+    <t>Pigment Implementation</t>
+  </si>
+  <si>
+    <t>Tim Callesen</t>
+  </si>
+  <si>
+    <t>Zareen Khan</t>
+  </si>
+  <si>
+    <t>Project/Client Name</t>
+  </si>
+  <si>
+    <t>Resource Level</t>
+  </si>
+  <si>
+    <t>Resource Skill Set</t>
+  </si>
+  <si>
+    <t>Start Date</t>
+  </si>
+  <si>
+    <t>End Date</t>
+  </si>
+  <si>
+    <t>Hours Per Week</t>
+  </si>
+  <si>
+    <t>Harrington Manufacturing – NetSuite ERP Implementation</t>
+  </si>
+  <si>
+    <t>Senior Consultant</t>
+  </si>
+  <si>
+    <t>04/01/2026</t>
+  </si>
+  <si>
+    <t>06/30/2026</t>
+  </si>
+  <si>
+    <t>Clearwater Retail – O2C Optimization</t>
+  </si>
+  <si>
     <t>Consultant</t>
   </si>
   <si>
-    <t>NetSuite - Record to Report</t>
-  </si>
-  <si>
-    <t>Bank Integration</t>
-  </si>
-  <si>
-    <t>P2P</t>
-  </si>
-  <si>
-    <t>Benjamin Liu</t>
+    <t>03/20/2026</t>
+  </si>
+  <si>
+    <t>05/31/2026</t>
+  </si>
+  <si>
+    <t>Pinnacle Logistics – Supply Chain Rollout</t>
+  </si>
+  <si>
+    <t>03/21/2026</t>
+  </si>
+  <si>
+    <t>06/27/2026</t>
+  </si>
+  <si>
+    <t>Meridian Financial – R2R Consolidation</t>
   </si>
   <si>
     <t>Manager</t>
   </si>
   <si>
-    <t>NetSuite - Procure to Pay</t>
-  </si>
-  <si>
-    <t>Accounting</t>
-  </si>
-  <si>
-    <t>R2R</t>
-  </si>
-  <si>
-    <t>Christine Chen</t>
-  </si>
-  <si>
-    <t>NetSuite - Order to Cash</t>
-  </si>
-  <si>
-    <t>NetSuite Implementation</t>
-  </si>
-  <si>
-    <t>Crystal Brent</t>
-  </si>
-  <si>
-    <t>Senior Consultant</t>
-  </si>
-  <si>
-    <t>NetSuite - Supply Chain</t>
-  </si>
-  <si>
-    <t>Delaney O'Neil</t>
-  </si>
-  <si>
-    <t>Pigment</t>
-  </si>
-  <si>
-    <t>Unassigned</t>
-  </si>
-  <si>
-    <t>Ethan Osborne</t>
-  </si>
-  <si>
-    <t>Phase 0</t>
-  </si>
-  <si>
-    <t>Grace Schwieters</t>
+    <t>05/01/2026</t>
+  </si>
+  <si>
+    <t>07/31/2026</t>
+  </si>
+  <si>
+    <t>Summit Healthcare – P2P Upgrade</t>
+  </si>
+  <si>
+    <t>04/15/2026</t>
+  </si>
+  <si>
+    <t>07/15/2026</t>
+  </si>
+  <si>
+    <t>Vantage Distribution – Full Suite Implementation</t>
+  </si>
+  <si>
+    <t>Apex Pharma – NetSuite Assessment</t>
+  </si>
+  <si>
+    <t>Senior Manager</t>
+  </si>
+  <si>
+    <t>05/15/2026</t>
+  </si>
+  <si>
+    <t>08/31/2026</t>
+  </si>
+  <si>
+    <t>Internal – Pre-Sales Support</t>
   </si>
   <si>
     <t>Analyst</t>
-  </si>
-  <si>
-    <t>Phase 1</t>
-  </si>
-  <si>
-    <t>Phase 0 Design</t>
-  </si>
-  <si>
-    <t>Hannah Imhoff</t>
-  </si>
-  <si>
-    <t>NS Implementation</t>
-  </si>
-  <si>
-    <t>O2C Analyst</t>
-  </si>
-  <si>
-    <t>Jake Johnsen</t>
-  </si>
-  <si>
-    <t>Julie Loiben</t>
-  </si>
-  <si>
-    <t>Flare</t>
-  </si>
-  <si>
-    <t>Katharine Yu</t>
-  </si>
-  <si>
-    <t>Lance Falk</t>
-  </si>
-  <si>
-    <t>Grub WBS</t>
-  </si>
-  <si>
-    <t>Lexie Dutch</t>
-  </si>
-  <si>
-    <t>Marcy Minnerly</t>
-  </si>
-  <si>
-    <t>Secondment</t>
-  </si>
-  <si>
-    <t>Mario DeFelice</t>
-  </si>
-  <si>
-    <t>Evaluation</t>
-  </si>
-  <si>
-    <t>ERP Evaluation</t>
-  </si>
-  <si>
-    <t>Melissa Cross</t>
-  </si>
-  <si>
-    <t>L2C Assessment</t>
-  </si>
-  <si>
-    <t>Assessment</t>
-  </si>
-  <si>
-    <t>Melissa Leighton</t>
-  </si>
-  <si>
-    <t>Neeraj Rajendran</t>
-  </si>
-  <si>
-    <t>Sui Foundation</t>
-  </si>
-  <si>
-    <t>Nick Hernandez</t>
-  </si>
-  <si>
-    <t>Nick Kolbow</t>
-  </si>
-  <si>
-    <t>Senior Manager</t>
-  </si>
-  <si>
-    <t>Ryan Artz</t>
-  </si>
-  <si>
-    <t>Arevon</t>
-  </si>
-  <si>
-    <t>BlankStreet Advisory</t>
-  </si>
-  <si>
-    <t>Procore Advisory</t>
-  </si>
-  <si>
-    <t>Operate</t>
-  </si>
-  <si>
-    <t>Sammy Latif</t>
-  </si>
-  <si>
-    <t>Shreyas Sampath</t>
-  </si>
-  <si>
-    <t>SuiteBilling Implementation</t>
-  </si>
-  <si>
-    <t>SuiteProjects Advisory</t>
-  </si>
-  <si>
-    <t>Pigment Implementation</t>
-  </si>
-  <si>
-    <t>Tim Callesen</t>
-  </si>
-  <si>
-    <t>Zareen Khan</t>
-  </si>
-  <si>
-    <t>Project/Client Name</t>
-  </si>
-  <si>
-    <t>Resource Level</t>
-  </si>
-  <si>
-    <t>Resource Skill Set</t>
-  </si>
-  <si>
-    <t>Start Date</t>
-  </si>
-  <si>
-    <t>End Date</t>
-  </si>
-  <si>
-    <t>Hours Per Week</t>
-  </si>
-  <si>
-    <t>Harrington Manufacturing – NetSuite ERP Implementation</t>
-  </si>
-  <si>
-    <t>04/01/2026</t>
-  </si>
-  <si>
-    <t>06/30/2026</t>
-  </si>
-  <si>
-    <t>Clearwater Retail – O2C Optimization</t>
-  </si>
-  <si>
-    <t>03/20/2026</t>
-  </si>
-  <si>
-    <t>05/31/2026</t>
-  </si>
-  <si>
-    <t>Pinnacle Logistics – Supply Chain Rollout</t>
-  </si>
-  <si>
-    <t>03/21/2026</t>
-  </si>
-  <si>
-    <t>06/27/2026</t>
-  </si>
-  <si>
-    <t>Meridian Financial – R2R Consolidation</t>
-  </si>
-  <si>
-    <t>05/01/2026</t>
-  </si>
-  <si>
-    <t>07/31/2026</t>
-  </si>
-  <si>
-    <t>Summit Healthcare – P2P Upgrade</t>
-  </si>
-  <si>
-    <t>04/15/2026</t>
-  </si>
-  <si>
-    <t>07/15/2026</t>
-  </si>
-  <si>
-    <t>Vantage Distribution – Full Suite Implementation</t>
-  </si>
-  <si>
-    <t>Apex Pharma – NetSuite Assessment</t>
-  </si>
-  <si>
-    <t>05/15/2026</t>
-  </si>
-  <si>
-    <t>08/31/2026</t>
-  </si>
-  <si>
-    <t>Internal – Pre-Sales Support</t>
   </si>
   <si>
     <t>05/30/2026</t>
@@ -917,14 +917,15 @@
       <c r="A2" t="s">
         <v>16</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" t="str">
+        <f>=VLOOKUP(A2,'Employee Master'!$A:$B,2,FALSE)</f>
+        <v>Consultant</v>
+      </c>
+      <c r="C2" t="s">
         <v>17</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>18</v>
-      </c>
-      <c r="D2" t="s">
-        <v>19</v>
       </c>
       <c r="E2" s="1">
         <v>0</v>
@@ -967,14 +968,15 @@
       <c r="A3" t="s">
         <v>16</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" t="str">
+        <f>=VLOOKUP(A3,'Employee Master'!$A:$B,2,FALSE)</f>
+        <v>Consultant</v>
+      </c>
+      <c r="C3" t="s">
         <v>17</v>
       </c>
-      <c r="C3" t="s">
-        <v>18</v>
-      </c>
       <c r="D3" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E3" s="3">
         <v>40</v>
@@ -1015,16 +1017,17 @@
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B4" t="str">
+        <f>=VLOOKUP(A4,'Employee Master'!$A:$B,2,FALSE)</f>
+        <v>Manager</v>
+      </c>
+      <c r="C4" t="s">
         <v>21</v>
       </c>
-      <c r="B4" t="s">
+      <c r="D4" t="s">
         <v>22</v>
-      </c>
-      <c r="C4" t="s">
-        <v>23</v>
-      </c>
-      <c r="D4" t="s">
-        <v>24</v>
       </c>
       <c r="E4" s="2">
         <v>20</v>
@@ -1065,16 +1068,17 @@
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>20</v>
+      </c>
+      <c r="B5" t="str">
+        <f>=VLOOKUP(A5,'Employee Master'!$A:$B,2,FALSE)</f>
+        <v>Manager</v>
+      </c>
+      <c r="C5" t="s">
         <v>21</v>
       </c>
-      <c r="B5" t="s">
-        <v>22</v>
-      </c>
-      <c r="C5" t="s">
+      <c r="D5" t="s">
         <v>23</v>
-      </c>
-      <c r="D5" t="s">
-        <v>25</v>
       </c>
       <c r="E5" s="2">
         <v>20</v>
@@ -1115,16 +1119,17 @@
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
+        <v>24</v>
+      </c>
+      <c r="B6" t="str">
+        <f>=VLOOKUP(A6,'Employee Master'!$A:$B,2,FALSE)</f>
+        <v>Manager</v>
+      </c>
+      <c r="C6" t="s">
+        <v>25</v>
+      </c>
+      <c r="D6" t="s">
         <v>26</v>
-      </c>
-      <c r="B6" t="s">
-        <v>22</v>
-      </c>
-      <c r="C6" t="s">
-        <v>27</v>
-      </c>
-      <c r="D6" t="s">
-        <v>28</v>
       </c>
       <c r="E6" s="3">
         <v>40</v>
@@ -1165,16 +1170,17 @@
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>29</v>
-      </c>
-      <c r="B7" t="s">
-        <v>30</v>
+        <v>27</v>
+      </c>
+      <c r="B7" t="str">
+        <f>=VLOOKUP(A7,'Employee Master'!$A:$B,2,FALSE)</f>
+        <v>Senior Consultant</v>
       </c>
       <c r="C7" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="D7" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="E7" s="3">
         <v>40</v>
@@ -1215,16 +1221,17 @@
     </row>
     <row r="8" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>32</v>
-      </c>
-      <c r="B8" t="s">
+        <v>29</v>
+      </c>
+      <c r="B8" t="str">
+        <f>=VLOOKUP(A8,'Employee Master'!$A:$B,2,FALSE)</f>
+        <v>Senior Consultant</v>
+      </c>
+      <c r="C8" t="s">
         <v>30</v>
       </c>
-      <c r="C8" t="s">
-        <v>33</v>
-      </c>
       <c r="D8" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="E8" s="3">
         <v>40</v>
@@ -1265,16 +1272,17 @@
     </row>
     <row r="9" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>35</v>
-      </c>
-      <c r="B9" t="s">
-        <v>30</v>
+        <v>32</v>
+      </c>
+      <c r="B9" t="str">
+        <f>=VLOOKUP(A9,'Employee Master'!$A:$B,2,FALSE)</f>
+        <v>Senior Consultant</v>
       </c>
       <c r="C9" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D9" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="E9" s="3">
         <v>40</v>
@@ -1315,16 +1323,17 @@
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>37</v>
-      </c>
-      <c r="B10" t="s">
-        <v>38</v>
+        <v>34</v>
+      </c>
+      <c r="B10" t="str">
+        <f>=VLOOKUP(A10,'Employee Master'!$A:$B,2,FALSE)</f>
+        <v>Analyst</v>
       </c>
       <c r="C10" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="D10" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="E10" s="1">
         <v>0</v>
@@ -1365,16 +1374,17 @@
     </row>
     <row r="11" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>37</v>
-      </c>
-      <c r="B11" t="s">
-        <v>38</v>
+        <v>34</v>
+      </c>
+      <c r="B11" t="str">
+        <f>=VLOOKUP(A11,'Employee Master'!$A:$B,2,FALSE)</f>
+        <v>Analyst</v>
       </c>
       <c r="C11" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="D11" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="E11" s="4">
         <v>45</v>
@@ -1415,16 +1425,17 @@
     </row>
     <row r="12" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>41</v>
-      </c>
-      <c r="B12" t="s">
+        <v>37</v>
+      </c>
+      <c r="B12" t="str">
+        <f>=VLOOKUP(A12,'Employee Master'!$A:$B,2,FALSE)</f>
+        <v>Analyst</v>
+      </c>
+      <c r="C12" t="s">
+        <v>25</v>
+      </c>
+      <c r="D12" t="s">
         <v>38</v>
-      </c>
-      <c r="C12" t="s">
-        <v>27</v>
-      </c>
-      <c r="D12" t="s">
-        <v>42</v>
       </c>
       <c r="E12" s="1">
         <v>0</v>
@@ -1465,16 +1476,17 @@
     </row>
     <row r="13" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>41</v>
-      </c>
-      <c r="B13" t="s">
-        <v>38</v>
+        <v>37</v>
+      </c>
+      <c r="B13" t="str">
+        <f>=VLOOKUP(A13,'Employee Master'!$A:$B,2,FALSE)</f>
+        <v>Analyst</v>
       </c>
       <c r="C13" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="D13" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E13" s="1">
         <v>0</v>
@@ -1515,16 +1527,17 @@
     </row>
     <row r="14" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>41</v>
-      </c>
-      <c r="B14" t="s">
-        <v>38</v>
+        <v>37</v>
+      </c>
+      <c r="B14" t="str">
+        <f>=VLOOKUP(A14,'Employee Master'!$A:$B,2,FALSE)</f>
+        <v>Analyst</v>
       </c>
       <c r="C14" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="D14" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="E14" s="3">
         <v>40</v>
@@ -1565,16 +1578,17 @@
     </row>
     <row r="15" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>44</v>
-      </c>
-      <c r="B15" t="s">
-        <v>22</v>
+        <v>40</v>
+      </c>
+      <c r="B15" t="str">
+        <f>=VLOOKUP(A15,'Employee Master'!$A:$B,2,FALSE)</f>
+        <v>Manager</v>
       </c>
       <c r="C15" t="s">
+        <v>28</v>
+      </c>
+      <c r="D15" t="s">
         <v>31</v>
-      </c>
-      <c r="D15" t="s">
-        <v>34</v>
       </c>
       <c r="E15" s="3">
         <v>40</v>
@@ -1615,16 +1629,17 @@
     </row>
     <row r="16" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>45</v>
-      </c>
-      <c r="B16" t="s">
-        <v>22</v>
+        <v>41</v>
+      </c>
+      <c r="B16" t="str">
+        <f>=VLOOKUP(A16,'Employee Master'!$A:$B,2,FALSE)</f>
+        <v>Manager</v>
       </c>
       <c r="C16" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="D16" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="E16" s="2">
         <v>5</v>
@@ -1665,16 +1680,17 @@
     </row>
     <row r="17" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>45</v>
-      </c>
-      <c r="B17" t="s">
-        <v>22</v>
+        <v>41</v>
+      </c>
+      <c r="B17" t="str">
+        <f>=VLOOKUP(A17,'Employee Master'!$A:$B,2,FALSE)</f>
+        <v>Manager</v>
       </c>
       <c r="C17" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="D17" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="E17" s="3">
         <v>40</v>
@@ -1715,16 +1731,17 @@
     </row>
     <row r="18" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>47</v>
-      </c>
-      <c r="B18" t="s">
-        <v>30</v>
+        <v>43</v>
+      </c>
+      <c r="B18" t="str">
+        <f>=VLOOKUP(A18,'Employee Master'!$A:$B,2,FALSE)</f>
+        <v>Senior Consultant</v>
       </c>
       <c r="C18" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D18" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="E18" s="3">
         <v>40</v>
@@ -1765,16 +1782,17 @@
     </row>
     <row r="19" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>48</v>
-      </c>
-      <c r="B19" t="s">
-        <v>38</v>
+        <v>44</v>
+      </c>
+      <c r="B19" t="str">
+        <f>=VLOOKUP(A19,'Employee Master'!$A:$B,2,FALSE)</f>
+        <v>Analyst</v>
       </c>
       <c r="C19" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="D19" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="E19" s="3">
         <v>40</v>
@@ -1815,16 +1833,17 @@
     </row>
     <row r="20" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>50</v>
-      </c>
-      <c r="B20" t="s">
-        <v>30</v>
+        <v>46</v>
+      </c>
+      <c r="B20" t="str">
+        <f>=VLOOKUP(A20,'Employee Master'!$A:$B,2,FALSE)</f>
+        <v>Senior Consultant</v>
       </c>
       <c r="C20" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="D20" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="E20" s="4">
         <v>45</v>
@@ -1865,16 +1884,17 @@
     </row>
     <row r="21" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>50</v>
-      </c>
-      <c r="B21" t="s">
-        <v>30</v>
+        <v>46</v>
+      </c>
+      <c r="B21" t="str">
+        <f>=VLOOKUP(A21,'Employee Master'!$A:$B,2,FALSE)</f>
+        <v>Senior Consultant</v>
       </c>
       <c r="C21" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="D21" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="E21" s="1">
         <v>0</v>
@@ -1915,16 +1935,17 @@
     </row>
     <row r="22" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>51</v>
-      </c>
-      <c r="B22" t="s">
-        <v>22</v>
+        <v>47</v>
+      </c>
+      <c r="B22" t="str">
+        <f>=VLOOKUP(A22,'Employee Master'!$A:$B,2,FALSE)</f>
+        <v>Manager</v>
       </c>
       <c r="C22" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="D22" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="E22" s="3">
         <v>40</v>
@@ -1965,16 +1986,17 @@
     </row>
     <row r="23" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>53</v>
-      </c>
-      <c r="B23" t="s">
-        <v>22</v>
+        <v>49</v>
+      </c>
+      <c r="B23" t="str">
+        <f>=VLOOKUP(A23,'Employee Master'!$A:$B,2,FALSE)</f>
+        <v>Manager</v>
       </c>
       <c r="C23" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="D23" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="E23" s="1">
         <v>0</v>
@@ -2015,16 +2037,17 @@
     </row>
     <row r="24" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>53</v>
-      </c>
-      <c r="B24" t="s">
-        <v>22</v>
+        <v>49</v>
+      </c>
+      <c r="B24" t="str">
+        <f>=VLOOKUP(A24,'Employee Master'!$A:$B,2,FALSE)</f>
+        <v>Manager</v>
       </c>
       <c r="C24" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="D24" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="E24" s="2">
         <v>16</v>
@@ -2065,16 +2088,17 @@
     </row>
     <row r="25" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>53</v>
-      </c>
-      <c r="B25" t="s">
-        <v>22</v>
+        <v>49</v>
+      </c>
+      <c r="B25" t="str">
+        <f>=VLOOKUP(A25,'Employee Master'!$A:$B,2,FALSE)</f>
+        <v>Manager</v>
       </c>
       <c r="C25" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="D25" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="E25" s="2">
         <v>8</v>
@@ -2115,16 +2139,17 @@
     </row>
     <row r="26" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>56</v>
-      </c>
-      <c r="B26" t="s">
-        <v>30</v>
+        <v>52</v>
+      </c>
+      <c r="B26" t="str">
+        <f>=VLOOKUP(A26,'Employee Master'!$A:$B,2,FALSE)</f>
+        <v>Senior Consultant</v>
       </c>
       <c r="C26" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D26" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="E26" s="2">
         <v>5</v>
@@ -2165,16 +2190,17 @@
     </row>
     <row r="27" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>56</v>
-      </c>
-      <c r="B27" t="s">
-        <v>30</v>
+        <v>52</v>
+      </c>
+      <c r="B27" t="str">
+        <f>=VLOOKUP(A27,'Employee Master'!$A:$B,2,FALSE)</f>
+        <v>Senior Consultant</v>
       </c>
       <c r="C27" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D27" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="E27" s="3">
         <v>40</v>
@@ -2215,16 +2241,17 @@
     </row>
     <row r="28" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>56</v>
-      </c>
-      <c r="B28" t="s">
-        <v>30</v>
+        <v>52</v>
+      </c>
+      <c r="B28" t="str">
+        <f>=VLOOKUP(A28,'Employee Master'!$A:$B,2,FALSE)</f>
+        <v>Senior Consultant</v>
       </c>
       <c r="C28" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D28" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="E28" s="1">
         <v>0</v>
@@ -2265,16 +2292,17 @@
     </row>
     <row r="29" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>59</v>
-      </c>
-      <c r="B29" t="s">
-        <v>22</v>
+        <v>55</v>
+      </c>
+      <c r="B29" t="str">
+        <f>=VLOOKUP(A29,'Employee Master'!$A:$B,2,FALSE)</f>
+        <v>Manager</v>
       </c>
       <c r="C29" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="D29" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="E29" s="3">
         <v>40</v>
@@ -2315,16 +2343,17 @@
     </row>
     <row r="30" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>60</v>
-      </c>
-      <c r="B30" t="s">
-        <v>38</v>
+        <v>56</v>
+      </c>
+      <c r="B30" t="str">
+        <f>=VLOOKUP(A30,'Employee Master'!$A:$B,2,FALSE)</f>
+        <v>Analyst</v>
       </c>
       <c r="C30" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="D30" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="E30" s="1">
         <v>0</v>
@@ -2365,16 +2394,17 @@
     </row>
     <row r="31" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>60</v>
-      </c>
-      <c r="B31" t="s">
-        <v>38</v>
+        <v>56</v>
+      </c>
+      <c r="B31" t="str">
+        <f>=VLOOKUP(A31,'Employee Master'!$A:$B,2,FALSE)</f>
+        <v>Analyst</v>
       </c>
       <c r="C31" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="D31" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="E31" s="3">
         <v>40</v>
@@ -2415,16 +2445,17 @@
     </row>
     <row r="32" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>62</v>
-      </c>
-      <c r="B32" t="s">
-        <v>30</v>
+        <v>58</v>
+      </c>
+      <c r="B32" t="str">
+        <f>=VLOOKUP(A32,'Employee Master'!$A:$B,2,FALSE)</f>
+        <v>Senior Consultant</v>
       </c>
       <c r="C32" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="D32" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="E32" s="1">
         <v>0</v>
@@ -2465,16 +2496,17 @@
     </row>
     <row r="33" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>62</v>
-      </c>
-      <c r="B33" t="s">
-        <v>30</v>
+        <v>58</v>
+      </c>
+      <c r="B33" t="str">
+        <f>=VLOOKUP(A33,'Employee Master'!$A:$B,2,FALSE)</f>
+        <v>Senior Consultant</v>
       </c>
       <c r="C33" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="D33" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="E33" s="3">
         <v>40</v>
@@ -2515,16 +2547,17 @@
     </row>
     <row r="34" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>63</v>
-      </c>
-      <c r="B34" t="s">
-        <v>64</v>
+        <v>59</v>
+      </c>
+      <c r="B34" t="str">
+        <f>=VLOOKUP(A34,'Employee Master'!$A:$B,2,FALSE)</f>
+        <v>Senior Manager</v>
       </c>
       <c r="C34" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="D34" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="E34" s="3">
         <v>40</v>
@@ -2565,16 +2598,17 @@
     </row>
     <row r="35" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>65</v>
-      </c>
-      <c r="B35" t="s">
-        <v>30</v>
+        <v>60</v>
+      </c>
+      <c r="B35" t="str">
+        <f>=VLOOKUP(A35,'Employee Master'!$A:$B,2,FALSE)</f>
+        <v>Senior Consultant</v>
       </c>
       <c r="C35" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D35" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="E35" s="2">
         <v>12</v>
@@ -2615,16 +2649,17 @@
     </row>
     <row r="36" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>65</v>
-      </c>
-      <c r="B36" t="s">
-        <v>30</v>
+        <v>60</v>
+      </c>
+      <c r="B36" t="str">
+        <f>=VLOOKUP(A36,'Employee Master'!$A:$B,2,FALSE)</f>
+        <v>Senior Consultant</v>
       </c>
       <c r="C36" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D36" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="E36" s="2">
         <v>20</v>
@@ -2665,16 +2700,17 @@
     </row>
     <row r="37" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>65</v>
-      </c>
-      <c r="B37" t="s">
-        <v>30</v>
+        <v>60</v>
+      </c>
+      <c r="B37" t="str">
+        <f>=VLOOKUP(A37,'Employee Master'!$A:$B,2,FALSE)</f>
+        <v>Senior Consultant</v>
       </c>
       <c r="C37" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D37" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="E37" s="2">
         <v>8</v>
@@ -2715,16 +2751,17 @@
     </row>
     <row r="38" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>65</v>
-      </c>
-      <c r="B38" t="s">
-        <v>30</v>
+        <v>60</v>
+      </c>
+      <c r="B38" t="str">
+        <f>=VLOOKUP(A38,'Employee Master'!$A:$B,2,FALSE)</f>
+        <v>Senior Consultant</v>
       </c>
       <c r="C38" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D38" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="E38" s="2">
         <v>4</v>
@@ -2765,16 +2802,17 @@
     </row>
     <row r="39" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>70</v>
-      </c>
-      <c r="B39" t="s">
-        <v>17</v>
+        <v>65</v>
+      </c>
+      <c r="B39" t="str">
+        <f>=VLOOKUP(A39,'Employee Master'!$A:$B,2,FALSE)</f>
+        <v>Consultant</v>
       </c>
       <c r="C39" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="D39" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="E39" s="3">
         <v>40</v>
@@ -2815,16 +2853,17 @@
     </row>
     <row r="40" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>71</v>
-      </c>
-      <c r="B40" t="s">
-        <v>22</v>
+        <v>66</v>
+      </c>
+      <c r="B40" t="str">
+        <f>=VLOOKUP(A40,'Employee Master'!$A:$B,2,FALSE)</f>
+        <v>Manager</v>
       </c>
       <c r="C40" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="D40" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="E40" s="2">
         <v>14</v>
@@ -2865,16 +2904,17 @@
     </row>
     <row r="41" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>71</v>
-      </c>
-      <c r="B41" t="s">
-        <v>22</v>
+        <v>66</v>
+      </c>
+      <c r="B41" t="str">
+        <f>=VLOOKUP(A41,'Employee Master'!$A:$B,2,FALSE)</f>
+        <v>Manager</v>
       </c>
       <c r="C41" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="D41" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="E41" s="2">
         <v>4</v>
@@ -2915,16 +2955,17 @@
     </row>
     <row r="42" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>71</v>
-      </c>
-      <c r="B42" t="s">
-        <v>22</v>
+        <v>66</v>
+      </c>
+      <c r="B42" t="str">
+        <f>=VLOOKUP(A42,'Employee Master'!$A:$B,2,FALSE)</f>
+        <v>Manager</v>
       </c>
       <c r="C42" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="D42" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="E42" s="2">
         <v>10</v>
@@ -2965,16 +3006,17 @@
     </row>
     <row r="43" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>71</v>
-      </c>
-      <c r="B43" t="s">
-        <v>22</v>
+        <v>66</v>
+      </c>
+      <c r="B43" t="str">
+        <f>=VLOOKUP(A43,'Employee Master'!$A:$B,2,FALSE)</f>
+        <v>Manager</v>
       </c>
       <c r="C43" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="D43" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="E43" s="2">
         <v>16</v>
@@ -3015,16 +3057,17 @@
     </row>
     <row r="44" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>75</v>
-      </c>
-      <c r="B44" t="s">
-        <v>64</v>
+        <v>70</v>
+      </c>
+      <c r="B44" t="str">
+        <f>=VLOOKUP(A44,'Employee Master'!$A:$B,2,FALSE)</f>
+        <v>Senior Manager</v>
       </c>
       <c r="C44" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="D44" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="E44" s="3">
         <v>40</v>
@@ -3065,16 +3108,17 @@
     </row>
     <row r="45" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>76</v>
-      </c>
-      <c r="B45" t="s">
-        <v>38</v>
+        <v>71</v>
+      </c>
+      <c r="B45" t="str">
+        <f>=VLOOKUP(A45,'Employee Master'!$A:$B,2,FALSE)</f>
+        <v>Analyst</v>
       </c>
       <c r="C45" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="D45" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="E45" s="2">
         <v>16</v>
@@ -3114,6 +3158,14 @@
       </c>
     </row>
   </sheetData>
+  <dataValidations count="2">
+    <dataValidation type="list" allowBlank="1" sqref="C2:C500">
+      <formula1>'Skills Master'!$A$2:$A$10</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" sqref="D2:D500">
+      <formula1>'Project Master'!$B$2:$B$27</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
@@ -3132,39 +3184,39 @@
   <sheetData>
     <row r="1" ht="30" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="E1" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="F1" s="5" t="s">
         <v>77</v>
-      </c>
-      <c r="B1" s="5" t="s">
-        <v>78</v>
-      </c>
-      <c r="C1" s="5" t="s">
-        <v>79</v>
-      </c>
-      <c r="D1" s="5" t="s">
-        <v>80</v>
-      </c>
-      <c r="E1" s="5" t="s">
-        <v>81</v>
-      </c>
-      <c r="F1" s="5" t="s">
-        <v>82</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>30</v>
+        <v>79</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D2" s="7" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="E2" s="7" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="F2" s="7">
         <v>40</v>
@@ -3172,19 +3224,19 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="B3" t="s">
-        <v>17</v>
+        <v>83</v>
       </c>
       <c r="C3" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="F3" s="8">
         <v>40</v>
@@ -3192,19 +3244,19 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>30</v>
+        <v>79</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="F4" s="7">
         <v>30</v>
@@ -3212,19 +3264,19 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>89</v>
+      </c>
+      <c r="B5" t="s">
+        <v>90</v>
+      </c>
+      <c r="C5" t="s">
+        <v>17</v>
+      </c>
+      <c r="D5" s="8" t="s">
+        <v>91</v>
+      </c>
+      <c r="E5" s="8" t="s">
         <v>92</v>
-      </c>
-      <c r="B5" t="s">
-        <v>22</v>
-      </c>
-      <c r="C5" t="s">
-        <v>18</v>
-      </c>
-      <c r="D5" s="8" t="s">
-        <v>93</v>
-      </c>
-      <c r="E5" s="8" t="s">
-        <v>94</v>
       </c>
       <c r="F5" s="8">
         <v>30</v>
@@ -3232,19 +3284,19 @@
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
+        <v>93</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="C6" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="E6" s="7" t="s">
         <v>95</v>
-      </c>
-      <c r="B6" s="6" t="s">
-        <v>30</v>
-      </c>
-      <c r="C6" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="D6" s="7" t="s">
-        <v>96</v>
-      </c>
-      <c r="E6" s="7" t="s">
-        <v>97</v>
       </c>
       <c r="F6" s="7">
         <v>40</v>
@@ -3252,19 +3304,19 @@
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="B7" t="s">
+        <v>83</v>
+      </c>
+      <c r="C7" t="s">
         <v>17</v>
       </c>
-      <c r="C7" t="s">
-        <v>18</v>
-      </c>
       <c r="D7" s="8" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="F7" s="8">
         <v>30</v>
@@ -3272,19 +3324,19 @@
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="B8" s="6" t="s">
+        <v>98</v>
+      </c>
+      <c r="C8" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="D8" s="7" t="s">
         <v>99</v>
       </c>
-      <c r="B8" s="6" t="s">
-        <v>64</v>
-      </c>
-      <c r="C8" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="D8" s="7" t="s">
+      <c r="E8" s="7" t="s">
         <v>100</v>
-      </c>
-      <c r="E8" s="7" t="s">
-        <v>101</v>
       </c>
       <c r="F8" s="7">
         <v>20</v>
@@ -3292,16 +3344,16 @@
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
+        <v>101</v>
+      </c>
+      <c r="B9" t="s">
         <v>102</v>
       </c>
-      <c r="B9" t="s">
-        <v>38</v>
-      </c>
       <c r="C9" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="D9" s="8" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="E9" s="8" t="s">
         <v>103</v>
@@ -3311,6 +3363,17 @@
       </c>
     </row>
   </sheetData>
+  <dataValidations count="3">
+    <dataValidation type="list" allowBlank="1" sqref="A2:A500">
+      <formula1>'Project Master'!$B$2:$B$27</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" sqref="B2:B500">
+      <formula1>'Resource Levels'!$A$2:$A$10</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" sqref="C2:C500">
+      <formula1>'Skills Master'!$A$2:$A$10</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
@@ -3338,199 +3401,199 @@
         <v>16</v>
       </c>
       <c r="B2" t="s">
-        <v>17</v>
+        <v>83</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B3" t="s">
-        <v>22</v>
+        <v>90</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B4" t="s">
-        <v>22</v>
+        <v>90</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="B5" t="s">
-        <v>30</v>
+        <v>79</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="B6" t="s">
-        <v>30</v>
+        <v>79</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="B7" t="s">
-        <v>30</v>
+        <v>79</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="B8" t="s">
-        <v>38</v>
+        <v>102</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="B9" t="s">
-        <v>38</v>
+        <v>102</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="B10" t="s">
-        <v>22</v>
+        <v>90</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="B11" t="s">
-        <v>22</v>
+        <v>90</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="B12" t="s">
-        <v>30</v>
+        <v>79</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="B13" t="s">
-        <v>38</v>
+        <v>102</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="B14" t="s">
-        <v>30</v>
+        <v>79</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="B15" t="s">
-        <v>22</v>
+        <v>90</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="B16" t="s">
-        <v>22</v>
+        <v>90</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="B17" t="s">
-        <v>30</v>
+        <v>79</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="B18" t="s">
-        <v>22</v>
+        <v>90</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="B19" t="s">
-        <v>38</v>
+        <v>102</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="B20" t="s">
-        <v>30</v>
+        <v>79</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="B21" t="s">
-        <v>64</v>
+        <v>98</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="B22" t="s">
-        <v>30</v>
+        <v>79</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="B23" t="s">
-        <v>17</v>
+        <v>83</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="B24" t="s">
-        <v>22</v>
+        <v>90</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="B25" t="s">
-        <v>64</v>
+        <v>98</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="B26" t="s">
-        <v>38</v>
+        <v>102</v>
       </c>
     </row>
   </sheetData>
@@ -3554,22 +3617,22 @@
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
     </row>
   </sheetData>
@@ -3593,27 +3656,27 @@
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>38</v>
+        <v>102</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>17</v>
+        <v>83</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>30</v>
+        <v>79</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>22</v>
+        <v>90</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>64</v>
+        <v>98</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
@@ -3649,7 +3712,7 @@
         <v>107</v>
       </c>
       <c r="B2" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
@@ -3657,7 +3720,7 @@
         <v>108</v>
       </c>
       <c r="B3" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -3665,7 +3728,7 @@
         <v>109</v>
       </c>
       <c r="B4" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
@@ -3673,7 +3736,7 @@
         <v>110</v>
       </c>
       <c r="B5" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
@@ -3681,7 +3744,7 @@
         <v>111</v>
       </c>
       <c r="B6" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
@@ -3689,7 +3752,7 @@
         <v>112</v>
       </c>
       <c r="B7" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
@@ -3697,7 +3760,7 @@
         <v>113</v>
       </c>
       <c r="B8" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
@@ -3705,7 +3768,7 @@
         <v>114</v>
       </c>
       <c r="B9" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
@@ -3713,7 +3776,7 @@
         <v>115</v>
       </c>
       <c r="B10" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
@@ -3721,7 +3784,7 @@
         <v>116</v>
       </c>
       <c r="B11" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
@@ -3729,7 +3792,7 @@
         <v>117</v>
       </c>
       <c r="B12" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
@@ -3737,7 +3800,7 @@
         <v>118</v>
       </c>
       <c r="B13" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
@@ -3745,7 +3808,7 @@
         <v>119</v>
       </c>
       <c r="B14" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
@@ -3753,7 +3816,7 @@
         <v>120</v>
       </c>
       <c r="B15" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
@@ -3761,7 +3824,7 @@
         <v>121</v>
       </c>
       <c r="B16" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
@@ -3769,7 +3832,7 @@
         <v>122</v>
       </c>
       <c r="B17" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
@@ -3777,7 +3840,7 @@
         <v>123</v>
       </c>
       <c r="B18" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
@@ -3785,7 +3848,7 @@
         <v>124</v>
       </c>
       <c r="B19" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
@@ -3793,7 +3856,7 @@
         <v>125</v>
       </c>
       <c r="B20" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
@@ -3801,7 +3864,7 @@
         <v>126</v>
       </c>
       <c r="B21" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
@@ -3809,7 +3872,7 @@
         <v>127</v>
       </c>
       <c r="B22" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.25">
@@ -3817,7 +3880,7 @@
         <v>128</v>
       </c>
       <c r="B23" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.25">
@@ -3825,7 +3888,7 @@
         <v>129</v>
       </c>
       <c r="B24" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.25">
@@ -3833,7 +3896,7 @@
         <v>130</v>
       </c>
       <c r="B25" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.25">
@@ -3841,7 +3904,7 @@
         <v>131</v>
       </c>
       <c r="B26" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.25">
@@ -3849,7 +3912,7 @@
         <v>132</v>
       </c>
       <c r="B27" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
     </row>
   </sheetData>

</xml_diff>